<commit_message>
Correccion de Codigos de cursos
</commit_message>
<xml_diff>
--- a/datos/Equivalencias_LLYA.xlsx
+++ b/datos/Equivalencias_LLYA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Consumo_horas_educacion_secundaria\datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD5B6277-125C-4260-A888-30B669BFB6BE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{819C922B-92B2-4AF5-9CD3-E0BB6A4ECFB3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1381,10 +1381,10 @@
         <v>15</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="I25" s="5">
         <v>5</v>

</xml_diff>